<commit_message>
Reorganize project items into 6 sub-categories in consolidated file
Splits 専案項目 40 items into A系統(14)/D系統(8)/K系統(1)/E系統(3)/會員平台(7)/其他(7) in column A.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026/2026單位目標績效表_全體整合.xlsx
+++ b/2026/2026單位目標績效表_全體整合.xlsx
@@ -1091,10 +1091,9 @@
       <c r="X5" s="49" t="n"/>
     </row>
     <row r="6" ht="41.5" customFormat="1" customHeight="1" s="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>專案項目
-(6)</t>
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>A系統</t>
         </is>
       </c>
       <c r="C6" s="56" t="inlineStr">
@@ -1135,7 +1134,7 @@
     <row r="7" ht="41.5" customFormat="1" customHeight="1" s="6">
       <c r="C7" s="56" t="inlineStr">
         <is>
-          <t>A系統-TWCA實名制(12月)</t>
+          <t>A/E/K系統-AWS(7月)</t>
         </is>
       </c>
       <c r="D7" s="48" t="n"/>
@@ -1146,7 +1145,7 @@
       <c r="I7" s="48" t="n"/>
       <c r="J7" s="49" t="n"/>
       <c r="K7" s="16" t="n">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="L7" s="49" t="n"/>
       <c r="M7" s="14" t="n"/>
@@ -1171,7 +1170,7 @@
     <row r="8" ht="41.5" customFormat="1" customHeight="1" s="6">
       <c r="C8" s="56" t="inlineStr">
         <is>
-          <t>D系統-秒殺自行選位(9月)</t>
+          <t>A系統-TWCA實名制(12月)</t>
         </is>
       </c>
       <c r="D8" s="48" t="n"/>
@@ -1207,7 +1206,7 @@
     <row r="9" ht="42.5" customFormat="1" customHeight="1" s="6">
       <c r="C9" s="56" t="inlineStr">
         <is>
-          <t>D系統-秒殺繼續選購(8月)</t>
+          <t>A系統-實名認證/實名制檢核(7~9月)</t>
         </is>
       </c>
       <c r="D9" s="48" t="n"/>
@@ -1218,7 +1217,7 @@
       <c r="I9" s="48" t="n"/>
       <c r="J9" s="49" t="n"/>
       <c r="K9" s="16" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="L9" s="49" t="n"/>
       <c r="M9" s="14" t="n"/>
@@ -1243,7 +1242,7 @@
     <row r="10" ht="43.5" customFormat="1" customHeight="1" s="6">
       <c r="C10" s="56" t="inlineStr">
         <is>
-          <t>A系統-svn版控轉移github(1月)</t>
+          <t>A系統-優化需求(12月)</t>
         </is>
       </c>
       <c r="D10" s="48" t="n"/>
@@ -1254,7 +1253,7 @@
       <c r="I10" s="48" t="n"/>
       <c r="J10" s="49" t="n"/>
       <c r="K10" s="16" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="L10" s="49" t="n"/>
       <c r="M10" s="15" t="n"/>
@@ -1279,7 +1278,7 @@
     <row r="11" ht="42" customFormat="1" customHeight="1" s="6">
       <c r="C11" s="56" t="inlineStr">
         <is>
-          <t>A系統-樂天桃猿APP需求(Phase II)(12月)</t>
+          <t>A系統-退票訂單by活動可選擇(12月)</t>
         </is>
       </c>
       <c r="D11" s="48" t="n"/>
@@ -1315,7 +1314,7 @@
     <row r="12" ht="42.5" customFormat="1" customHeight="1" s="6">
       <c r="C12" s="56" t="inlineStr">
         <is>
-          <t>A系統-退票訂單by活動可選擇(12月)</t>
+          <t>A系統-退票相關(11月)</t>
         </is>
       </c>
       <c r="D12" s="48" t="n"/>
@@ -1326,7 +1325,7 @@
       <c r="I12" s="48" t="n"/>
       <c r="J12" s="49" t="n"/>
       <c r="K12" s="16" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="L12" s="49" t="n"/>
       <c r="M12" s="14" t="n"/>
@@ -1351,7 +1350,7 @@
     <row r="13" ht="44" customFormat="1" customHeight="1" s="6">
       <c r="C13" s="56" t="inlineStr">
         <is>
-          <t>A系統-票卡需求phase I(12月)</t>
+          <t>A系統-樂天桃猿APP需求(Phase II)(12月)</t>
         </is>
       </c>
       <c r="D13" s="48" t="n"/>
@@ -1387,7 +1386,7 @@
     <row r="14" ht="43" customFormat="1" customHeight="1" s="6">
       <c r="C14" s="56" t="inlineStr">
         <is>
-          <t>K系統-離峰班次回傳指定agent id(12月)</t>
+          <t>A系統-票卡需求phase I(12月)</t>
         </is>
       </c>
       <c r="D14" s="48" t="n"/>
@@ -1398,7 +1397,7 @@
       <c r="I14" s="48" t="n"/>
       <c r="J14" s="49" t="n"/>
       <c r="K14" s="16" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="L14" s="49" t="n"/>
       <c r="M14" s="14" t="n"/>
@@ -1423,7 +1422,7 @@
     <row r="15" ht="42.5" customFormat="1" customHeight="1" s="6">
       <c r="C15" s="56" t="inlineStr">
         <is>
-          <t>A系統-限制同時多裝置操作購票(12月)</t>
+          <t>A系統-svn版控轉移github(1月)</t>
         </is>
       </c>
       <c r="D15" s="48" t="n"/>
@@ -1434,7 +1433,7 @@
       <c r="I15" s="48" t="n"/>
       <c r="J15" s="49" t="n"/>
       <c r="K15" s="16" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="L15" s="49" t="n"/>
       <c r="M15" s="14" t="n"/>
@@ -1459,7 +1458,7 @@
     <row r="16" ht="30.5" customFormat="1" customHeight="1" s="6">
       <c r="C16" s="56" t="inlineStr">
         <is>
-          <t>A系統-後台活動埋廠商GA追蹤碼設定功能(12月)</t>
+          <t>A系統-限制同時多裝置操作購票(12月)</t>
         </is>
       </c>
       <c r="D16" s="48" t="n"/>
@@ -1470,7 +1469,7 @@
       <c r="I16" s="48" t="n"/>
       <c r="J16" s="49" t="n"/>
       <c r="K16" s="16" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="L16" s="49" t="n"/>
       <c r="M16" s="14" t="n"/>
@@ -1495,7 +1494,7 @@
     <row r="17" ht="44" customFormat="1" customHeight="1" s="6">
       <c r="C17" s="56" t="inlineStr">
         <is>
-          <t>AI應用-研究OCC/ORS重構(12月)</t>
+          <t>A系統-後台活動埋廠商GA追蹤碼設定功能(12月)</t>
         </is>
       </c>
       <c r="D17" s="48" t="n"/>
@@ -1506,7 +1505,7 @@
       <c r="I17" s="48" t="n"/>
       <c r="J17" s="49" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="L17" s="49" t="n"/>
       <c r="M17" s="14" t="n"/>
@@ -1531,7 +1530,7 @@
     <row r="18" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C18" s="56" t="inlineStr">
         <is>
-          <t>優化-OCC/ORS反組譯程式重建(12月)</t>
+          <t>AI應用-研究OCC/ORS重構(12月)</t>
         </is>
       </c>
       <c r="D18" s="48" t="n"/>
@@ -1567,7 +1566,7 @@
     <row r="19" ht="17" customFormat="1" customHeight="1" s="6">
       <c r="C19" s="56" t="inlineStr">
         <is>
-          <t>A/E/K系統-AWS(7月)</t>
+          <t>優化-OCC/ORS反組譯程式重建(12月)</t>
         </is>
       </c>
       <c r="D19" s="48" t="n"/>
@@ -1578,7 +1577,7 @@
       <c r="I19" s="48" t="n"/>
       <c r="J19" s="49" t="n"/>
       <c r="K19" s="16" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="L19" s="49" t="n"/>
       <c r="M19" s="14" t="n"/>
@@ -1601,9 +1600,14 @@
       <c r="X19" s="49" t="n"/>
     </row>
     <row r="20" ht="30" customFormat="1" customHeight="1" s="6">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>D系統</t>
+        </is>
+      </c>
       <c r="C20" s="33" t="inlineStr">
         <is>
-          <t>A系統-實名認證/實名制檢核(7~9月)</t>
+          <t>D系統-秒殺自行選位(9月)</t>
         </is>
       </c>
       <c r="D20" s="48" t="n"/>
@@ -1614,7 +1618,7 @@
       <c r="I20" s="48" t="n"/>
       <c r="J20" s="49" t="n"/>
       <c r="K20" s="13" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="L20" s="49" t="n"/>
       <c r="M20" s="35" t="n"/>
@@ -1639,7 +1643,7 @@
     <row r="21" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C21" s="33" t="inlineStr">
         <is>
-          <t>A系統-優化需求(12月)</t>
+          <t>D系統-秒殺繼續選購(8月)</t>
         </is>
       </c>
       <c r="D21" s="48" t="n"/>
@@ -1650,7 +1654,7 @@
       <c r="I21" s="48" t="n"/>
       <c r="J21" s="49" t="n"/>
       <c r="K21" s="13" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="L21" s="49" t="n"/>
       <c r="M21" s="55" t="n"/>
@@ -1675,7 +1679,7 @@
     <row r="22" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C22" s="33" t="inlineStr">
         <is>
-          <t>A系統-退票相關(11月)</t>
+          <t>D系統-DB轉AWS(5月)</t>
         </is>
       </c>
       <c r="D22" s="48" t="n"/>
@@ -1686,7 +1690,7 @@
       <c r="I22" s="48" t="n"/>
       <c r="J22" s="49" t="n"/>
       <c r="K22" s="13" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="L22" s="49" t="n"/>
       <c r="M22" s="35" t="n"/>
@@ -1711,7 +1715,7 @@
     <row r="23" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>E系統-主辦權限優化(7月)</t>
+          <t>D系統-社群歸戶(1-2月)</t>
         </is>
       </c>
       <c r="K23" s="4" t="n">
@@ -1732,19 +1736,19 @@
     <row r="24" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>E系統-方案庫存(4月)</t>
+          <t>D系統移轉PostgreSQL(5月上線)</t>
         </is>
       </c>
       <c r="K24" s="4" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="M24" s="4" t="n"/>
       <c r="U24" s="4" t="n"/>
-      <c r="V24">
+      <c r="V24" s="0">
         <f>CODE(U24)</f>
         <v/>
       </c>
-      <c r="W24">
+      <c r="W24" s="0">
         <f>CHOOSE(V24-64,5,4.75,4.5,4.25,4)*K24</f>
         <v/>
       </c>
@@ -1752,11 +1756,11 @@
     <row r="25" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>E系統-ESIM卡(5月)</t>
+          <t>D系統AWS Log費用減量規畫(5月上線)</t>
         </is>
       </c>
       <c r="K25" s="4" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="M25" s="4" t="n"/>
       <c r="U25" s="4" t="n"/>
@@ -1772,11 +1776,11 @@
     <row r="26" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>D系統-DB轉AWS(5月)</t>
+          <t>D系統_會員必須先登功能(Q2)</t>
         </is>
       </c>
       <c r="K26" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="M26" s="4" t="n"/>
       <c r="U26" s="4" t="n"/>
@@ -1792,11 +1796,11 @@
     <row r="27" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>A/E系統-OP兌點(12月)</t>
+          <t>優化-D系統導入CI/CD部署流程</t>
         </is>
       </c>
       <c r="K27" s="4" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="M27" s="4" t="n"/>
       <c r="U27" s="4" t="n"/>
@@ -1810,13 +1814,18 @@
       </c>
     </row>
     <row r="28" ht="14.5" customFormat="1" customHeight="1" s="6">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>K系統</t>
+        </is>
+      </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Q系統-2.1G(12月)</t>
+          <t>K系統-離峰班次回傳指定agent id(12月)</t>
         </is>
       </c>
       <c r="K28" s="4" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="M28" s="4" t="n"/>
       <c r="U28" s="4" t="n"/>
@@ -1830,13 +1839,18 @@
       </c>
     </row>
     <row r="29" ht="14.5" customFormat="1" customHeight="1" s="6">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>E系統</t>
+        </is>
+      </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>社群會員平台_社群登入_服務平台化Phase1 (2026/Q1)</t>
+          <t>E系統-主辦權限優化(7月)</t>
         </is>
       </c>
       <c r="K29" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M29" s="4" t="n"/>
       <c r="U29" s="4" t="n"/>
@@ -1852,11 +1866,11 @@
     <row r="30" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>社群會員平台_社群登入_會員手機TWCA身份認證(Q4)</t>
+          <t>E系統-方案庫存(4月)</t>
         </is>
       </c>
       <c r="K30" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="M30" s="4" t="n"/>
       <c r="U30" s="4" t="n"/>
@@ -1872,11 +1886,11 @@
     <row r="31" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>社群會員平台_社群登入_i禮讚APP串接(Q2)</t>
+          <t>E系統-ESIM卡(5月)</t>
         </is>
       </c>
       <c r="K31" s="4" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="M31" s="4" t="n"/>
       <c r="U31" s="4" t="n"/>
@@ -1890,9 +1904,14 @@
       </c>
     </row>
     <row r="32" ht="14.5" customFormat="1" customHeight="1" s="6">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>會員平台</t>
+        </is>
+      </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>社群會員平台_社群登入_海外電信提供手動產OTP機制(Q2)</t>
+          <t>社群會員平台_社群登入_服務平台化Phase1 (2026/Q1)</t>
         </is>
       </c>
       <c r="K32" s="4" t="n">
@@ -1912,11 +1931,11 @@
     <row r="33" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>社群會員平台_社群登入_優化已連動的手機號碼須再輸入登入密碼(Q2)</t>
+          <t>社群會員平台_社群登入_會員手機TWCA身份認證(Q4)</t>
         </is>
       </c>
       <c r="K33" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M33" s="4" t="n"/>
       <c r="U33" s="4" t="n"/>
@@ -1932,7 +1951,7 @@
     <row r="34" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>社群會員平台_社群登入_Email修改需驗證(Q2)</t>
+          <t>社群會員平台_社群登入_i禮讚APP串接(Q2)</t>
         </is>
       </c>
       <c r="K34" s="4" t="n">
@@ -1952,11 +1971,11 @@
     <row r="35" ht="14.5" customFormat="1" customHeight="1" s="6">
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>D系統_會員必須先登功能(Q2)</t>
+          <t>社群會員平台_社群登入_海外電信提供手動產OTP機制(Q2)</t>
         </is>
       </c>
       <c r="K35" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M35" s="4" t="n"/>
       <c r="U35" s="4" t="n"/>
@@ -1972,7 +1991,7 @@
     <row r="36">
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>社群會員平台_優化_OP點數平台新增查詢介面提供雲端卡反查功能</t>
+          <t>社群會員平台_社群登入_優化已連動的手機號碼須再輸入登入密碼(Q2)</t>
         </is>
       </c>
       <c r="K36" s="4" t="n">
@@ -1992,7 +2011,7 @@
     <row r="37">
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>AI運用_Queueit排隊自動設定</t>
+          <t>社群會員平台_社群登入_Email修改需驗證(Q2)</t>
         </is>
       </c>
       <c r="K37" s="4" t="n">
@@ -2010,414 +2029,419 @@
       </c>
     </row>
     <row r="38">
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>D系統-社群歸戶(1-2月)</t>
-        </is>
-      </c>
-      <c r="K38" t="n">
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>社群會員平台_優化_OP點數平台新增查詢介面提供雲端卡反查功能</t>
+        </is>
+      </c>
+      <c r="K38" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="V38">
+      <c r="V38" s="0">
         <f>CODE(U38)</f>
         <v/>
       </c>
-      <c r="W38">
+      <c r="W38" s="0">
         <f>CHOOSE(V38-64,5,4.75,4.5,4.25,4)*K38</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>D系統移轉PostgreSQL(5月上線)</t>
-        </is>
-      </c>
-      <c r="K39" t="n">
-        <v>2</v>
-      </c>
-      <c r="V39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>A/E系統-OP兌點(12月)</t>
+        </is>
+      </c>
+      <c r="K39" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V39" s="0">
         <f>CODE(U39)</f>
         <v/>
       </c>
-      <c r="W39">
+      <c r="W39" s="0">
         <f>CHOOSE(V39-64,5,4.75,4.5,4.25,4)*K39</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>D系統AWS Log費用減量規畫(5月上線)</t>
-        </is>
-      </c>
-      <c r="K40" t="n">
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Q系統-2.1G(12月)</t>
+        </is>
+      </c>
+      <c r="K40" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V40" s="0">
+        <f>CODE(U40)</f>
+        <v/>
+      </c>
+      <c r="W40" s="0">
+        <f>CHOOSE(V40-64,5,4.75,4.5,4.25,4)*K40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>AI運用_Queueit排隊自動設定</t>
+        </is>
+      </c>
+      <c r="K41" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="V40">
-        <f>CODE(U40)</f>
-        <v/>
-      </c>
-      <c r="W40">
-        <f>CHOOSE(V40-64,5,4.75,4.5,4.25,4)*K40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="C41" t="inlineStr">
+      <c r="V41" s="0">
+        <f>CODE(U41)</f>
+        <v/>
+      </c>
+      <c r="W41" s="0">
+        <f>CHOOSE(V41-64,5,4.75,4.5,4.25,4)*K41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>Predata改版(A/E/D)</t>
         </is>
       </c>
-      <c r="K41" t="n">
+      <c r="K42" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="V41">
-        <f>CODE(U41)</f>
-        <v/>
-      </c>
-      <c r="W41">
-        <f>CHOOSE(V41-64,5,4.75,4.5,4.25,4)*K41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="C42" t="inlineStr">
+      <c r="V42" s="0">
+        <f>CODE(U42)</f>
+        <v/>
+      </c>
+      <c r="W42" s="0">
+        <f>CHOOSE(V42-64,5,4.75,4.5,4.25,4)*K42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>Azure FrontDoor 升級(禮贈/會員)(8月-9月)</t>
         </is>
       </c>
-      <c r="K42" t="n">
+      <c r="K43" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="V42">
-        <f>CODE(U42)</f>
-        <v/>
-      </c>
-      <c r="W42">
-        <f>CHOOSE(V42-64,5,4.75,4.5,4.25,4)*K42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="C43" t="inlineStr">
+      <c r="V43" s="0">
+        <f>CODE(U43)</f>
+        <v/>
+      </c>
+      <c r="W43" s="0">
+        <f>CHOOSE(V43-64,5,4.75,4.5,4.25,4)*K43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>雲端主機EDR 導入CrowdStrike</t>
         </is>
       </c>
-      <c r="K43" t="n">
+      <c r="K44" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="V43">
-        <f>CODE(U43)</f>
-        <v/>
-      </c>
-      <c r="W43">
-        <f>CHOOSE(V43-64,5,4.75,4.5,4.25,4)*K43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>優化-D系統導入CI/CD部署流程</t>
-        </is>
-      </c>
-      <c r="K44" t="n">
+      <c r="V44" s="0">
+        <f>CODE(U44)</f>
+        <v/>
+      </c>
+      <c r="W44" s="0">
+        <f>CHOOSE(V44-64,5,4.75,4.5,4.25,4)*K44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>AI-協助系統Log分析與查詢</t>
+        </is>
+      </c>
+      <c r="K45" s="0" t="n">
         <v>0.25</v>
       </c>
-      <c r="V44">
-        <f>CODE(U44)</f>
-        <v/>
-      </c>
-      <c r="W44">
-        <f>CHOOSE(V44-64,5,4.75,4.5,4.25,4)*K44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>AI-協助系統Log分析與查詢</t>
-        </is>
-      </c>
-      <c r="K45" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="V45">
+      <c r="V45" s="0">
         <f>CODE(U45)</f>
         <v/>
       </c>
-      <c r="W45">
+      <c r="W45" s="0">
         <f>CHOOSE(V45-64,5,4.75,4.5,4.25,4)*K45</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="0" t="inlineStr">
         <is>
           <t>維運平台
 (2)</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>A系統_維運協助(進度管理/系統檢討修改/調整/障礙確認)</t>
         </is>
       </c>
-      <c r="K46" t="n">
+      <c r="K46" s="0" t="n">
         <v>1.5</v>
       </c>
-      <c r="V46">
+      <c r="V46" s="0">
         <f>CODE(U46)</f>
         <v/>
       </c>
-      <c r="W46">
+      <c r="W46" s="0">
         <f>CHOOSE(V46-64,5,4.75,4.5,4.25,4)*K46</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>K系統_維運協助(進度管理/系統檢討修改/調整/障礙確認)</t>
         </is>
       </c>
-      <c r="K47" t="n">
+      <c r="K47" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="V47">
+      <c r="V47" s="0">
         <f>CODE(U47)</f>
         <v/>
       </c>
-      <c r="W47">
+      <c r="W47" s="0">
         <f>CHOOSE(V47-64,5,4.75,4.5,4.25,4)*K47</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>Qware售票系統(A/C/D/Q/E)_維運協助(進度管理/系統檢討修改/調整/障礙確認)</t>
         </is>
       </c>
-      <c r="K48" t="n">
+      <c r="K48" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="V48">
+      <c r="V48" s="0">
         <f>CODE(U48)</f>
         <v/>
       </c>
-      <c r="W48">
+      <c r="W48" s="0">
         <f>CHOOSE(V48-64,5,4.75,4.5,4.25,4)*K48</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>A/E系統(需求訪談/整體架構規劃/障礙確認)</t>
         </is>
       </c>
-      <c r="K49" t="n">
+      <c r="K49" s="0" t="n">
         <v>0.8</v>
       </c>
-      <c r="V49">
+      <c r="V49" s="0">
         <f>CODE(U49)</f>
         <v/>
       </c>
-      <c r="W49">
+      <c r="W49" s="0">
         <f>CHOOSE(V49-64,5,4.75,4.5,4.25,4)*K49</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>其它專案(需求訪談/整體架構規劃/障礙確認)</t>
         </is>
       </c>
-      <c r="K50" t="n">
+      <c r="K50" s="0" t="n">
         <v>0.2</v>
       </c>
-      <c r="V50">
+      <c r="V50" s="0">
         <f>CODE(U50)</f>
         <v/>
       </c>
-      <c r="W50">
+      <c r="W50" s="0">
         <f>CHOOSE(V50-64,5,4.75,4.5,4.25,4)*K50</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>Qware售票系統(A)_維運協助(進度管理/系統檢討修改/調整/障礙確認)</t>
         </is>
       </c>
-      <c r="K51" t="n">
+      <c r="K51" s="0" t="n">
         <v>0.75</v>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="M51" s="0" t="inlineStr">
         <is>
           <t>(1)依需求緊急程度進行各項工作排定、品質控管，且進度能如期達成
 (2)確實執行障礙的調查及管理</t>
         </is>
       </c>
-      <c r="V51">
+      <c r="V51" s="0">
         <f>CODE(U51)</f>
         <v/>
       </c>
-      <c r="W51">
+      <c r="W51" s="0">
         <f>CHOOSE(V51-64,5,4.75,4.5,4.25,4)*K51</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="0" t="inlineStr">
         <is>
           <t>社群會員平台(需求訪談/整體架構規劃/障礙確認)</t>
         </is>
       </c>
-      <c r="K52" t="n">
+      <c r="K52" s="0" t="n">
         <v>0.75</v>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="M52" s="0" t="inlineStr">
         <is>
           <t>依需求的緊急需要，進行訪談匯整及對外包商進行需求的提出、進度管理。</t>
         </is>
       </c>
-      <c r="V52">
+      <c r="V52" s="0">
         <f>CODE(U52)</f>
         <v/>
       </c>
-      <c r="W52">
+      <c r="W52" s="0">
         <f>CHOOSE(V52-64,5,4.75,4.5,4.25,4)*K52</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="0" t="inlineStr">
         <is>
           <t>各平台相關報告</t>
         </is>
       </c>
-      <c r="K53" t="n">
+      <c r="K53" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="M53" s="0" t="inlineStr">
         <is>
           <t>依負責的平台，於會議進行說明報告</t>
         </is>
       </c>
-      <c r="V53">
+      <c r="V53" s="0">
         <f>CODE(U53)</f>
         <v/>
       </c>
-      <c r="W53">
+      <c r="W53" s="0">
         <f>CHOOSE(V53-64,5,4.75,4.5,4.25,4)*K53</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="0" t="inlineStr">
         <is>
           <t>Qware售票系統(A/D/E/球團App)_維運協助(進度管理/系統檢討修改/調整/障礙確認)</t>
         </is>
       </c>
-      <c r="K54" t="n">
+      <c r="K54" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="V54">
+      <c r="V54" s="0">
         <f>CODE(U54)</f>
         <v/>
       </c>
-      <c r="W54">
+      <c r="W54" s="0">
         <f>CHOOSE(V54-64,5,4.75,4.5,4.25,4)*K54</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="0" t="inlineStr">
         <is>
           <t>D系統(需求訪談/整體架構規劃/障礙確認)</t>
         </is>
       </c>
-      <c r="K55" t="n">
+      <c r="K55" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="M55" s="0" t="inlineStr">
         <is>
           <t>Queue-it 調整Aws 服務串接實作
 線上購票會員登入檢查機制</t>
         </is>
       </c>
-      <c r="V55">
+      <c r="V55" s="0">
         <f>CODE(U55)</f>
         <v/>
       </c>
-      <c r="W55">
+      <c r="W55" s="0">
         <f>CHOOSE(V55-64,5,4.75,4.5,4.25,4)*K55</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="0" t="inlineStr">
         <is>
           <t>雲端平台(日常維運、架構管理、障礙支援)</t>
         </is>
       </c>
-      <c r="K56" t="n">
+      <c r="K56" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="M56" s="0" t="inlineStr">
         <is>
           <t>導入 AWS 原生安全服務(GuardDuty/Security Hub)</t>
         </is>
       </c>
-      <c r="V56">
+      <c r="V56" s="0">
         <f>CODE(U56)</f>
         <v/>
       </c>
-      <c r="W56">
+      <c r="W56" s="0">
         <f>CHOOSE(V56-64,5,4.75,4.5,4.25,4)*K56</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="0" t="inlineStr">
         <is>
           <t>加分項目</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="0" t="inlineStr">
         <is>
           <t>提案(依據經營企劃通報獎勵辦法)，由基本獎至重大貢獻獎依序總分加分為 0.5、0.5、0.75、1、1.25</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="0" t="inlineStr">
         <is>
           <t>Team專案列表</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="0" t="inlineStr">
         <is>
           <t>專利申請 (提出 : 總分+ 0.5 ， 申請通過: 總分+ 0.5  )</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="W60">
+      <c r="W60" s="0">
         <f>SUM(W4:X59)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="244">
+  <mergeCells count="249">
     <mergeCell ref="M53:T53"/>
     <mergeCell ref="W4:X4"/>
     <mergeCell ref="K49:L49"/>
@@ -2451,12 +2475,12 @@
     <mergeCell ref="W43:X43"/>
     <mergeCell ref="C59:J59"/>
     <mergeCell ref="M6:T6"/>
+    <mergeCell ref="A20:B27"/>
     <mergeCell ref="C11:J11"/>
     <mergeCell ref="M15:T15"/>
+    <mergeCell ref="C46:J46"/>
     <mergeCell ref="M28:T28"/>
-    <mergeCell ref="A6:B45"/>
     <mergeCell ref="K42:L42"/>
-    <mergeCell ref="C46:J46"/>
     <mergeCell ref="M37:T37"/>
     <mergeCell ref="C52:J52"/>
     <mergeCell ref="W42:X42"/>
@@ -2469,6 +2493,7 @@
     <mergeCell ref="M14:T14"/>
     <mergeCell ref="K28:L28"/>
     <mergeCell ref="M29:T29"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="M23:T23"/>
     <mergeCell ref="K37:L37"/>
     <mergeCell ref="W14:X14"/>
@@ -2502,6 +2527,7 @@
     <mergeCell ref="M54:T54"/>
     <mergeCell ref="W54:X54"/>
     <mergeCell ref="W32:X32"/>
+    <mergeCell ref="A39:B45"/>
     <mergeCell ref="C55:J55"/>
     <mergeCell ref="W41:X41"/>
     <mergeCell ref="C9:J9"/>
@@ -2536,8 +2562,8 @@
     <mergeCell ref="M19:T19"/>
     <mergeCell ref="C37:J37"/>
     <mergeCell ref="K6:L6"/>
+    <mergeCell ref="W19:X19"/>
     <mergeCell ref="C18:J18"/>
-    <mergeCell ref="W19:X19"/>
     <mergeCell ref="S2:U2"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="W44:X44"/>
@@ -2587,8 +2613,8 @@
     <mergeCell ref="W21:X21"/>
     <mergeCell ref="C27:J27"/>
     <mergeCell ref="M27:T27"/>
+    <mergeCell ref="K23:L23"/>
     <mergeCell ref="W13:X13"/>
-    <mergeCell ref="K23:L23"/>
     <mergeCell ref="M36:T36"/>
     <mergeCell ref="M18:T18"/>
     <mergeCell ref="M45:T45"/>
@@ -2598,7 +2624,9 @@
     <mergeCell ref="C17:J17"/>
     <mergeCell ref="K7:L7"/>
     <mergeCell ref="M8:T8"/>
+    <mergeCell ref="A29:B31"/>
     <mergeCell ref="K57:L57"/>
+    <mergeCell ref="A32:B38"/>
     <mergeCell ref="C19:J19"/>
     <mergeCell ref="C53:J53"/>
     <mergeCell ref="K18:L18"/>
@@ -2624,6 +2652,7 @@
     <mergeCell ref="C29:J29"/>
     <mergeCell ref="A1:F2"/>
     <mergeCell ref="C47:J47"/>
+    <mergeCell ref="A6:B19"/>
     <mergeCell ref="C44:J44"/>
     <mergeCell ref="C22:J22"/>
     <mergeCell ref="K22:L22"/>
@@ -2632,9 +2661,9 @@
     <mergeCell ref="M40:T40"/>
     <mergeCell ref="C12:J12"/>
     <mergeCell ref="K59:L59"/>
+    <mergeCell ref="K12:L12"/>
     <mergeCell ref="C21:J21"/>
     <mergeCell ref="U3:V3"/>
-    <mergeCell ref="K12:L12"/>
     <mergeCell ref="M12:T12"/>
     <mergeCell ref="C51:J51"/>
     <mergeCell ref="M21:T21"/>

</xml_diff>